<commit_message>
Ajuste a módulo Desiertas, y al módulo Intro
</commit_message>
<xml_diff>
--- a/data/CATALOGO_LCA.xlsx
+++ b/data/CATALOGO_LCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d52177a9150211f7/rubrica_ENES_Merida/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="11_254BBF17CC517BB5C031F8B840107E71CFCECBAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF215B95-7DB9-4F28-B5F2-8C70B7D7E7FA}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_254BBF17CC517BB5C031F8B840107E71CFCECBAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49EB08A2-5531-483A-ACF2-CF4773B3EAAF}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3990" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANES 2022-2026" sheetId="1" r:id="rId1"/>
@@ -1635,9 +1635,6 @@
     <t>Químico, Ingeniero Químico, Ambiental, Civil o Biólogo.</t>
   </si>
   <si>
-    <t>aisgnatura</t>
-  </si>
-  <si>
     <t>semestre_grupo</t>
   </si>
   <si>
@@ -1657,6 +1654,9 @@
   </si>
   <si>
     <t>LCA, semestres 5° y 7° (optativas)</t>
+  </si>
+  <si>
+    <t>asignatura</t>
   </si>
 </sst>
 </file>
@@ -19707,7 +19707,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="11" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>49</v>
@@ -19716,12 +19716,12 @@
         <v>50</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>58</v>
@@ -19736,7 +19736,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>62</v>
@@ -19751,7 +19751,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>64</v>
@@ -19766,7 +19766,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>68</v>
@@ -19781,7 +19781,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>70</v>
@@ -19796,7 +19796,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>66</v>
@@ -19811,7 +19811,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>73</v>
@@ -19826,7 +19826,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>58</v>
@@ -19841,7 +19841,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>62</v>
@@ -19856,7 +19856,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B11" s="12" t="s">
         <v>64</v>
@@ -19871,7 +19871,7 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>68</v>
@@ -19886,7 +19886,7 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>70</v>
@@ -19901,7 +19901,7 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B14" s="12" t="s">
         <v>66</v>
@@ -19916,7 +19916,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>73</v>
@@ -19931,7 +19931,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B16" s="12" t="s">
         <v>89</v>
@@ -19946,7 +19946,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B17" s="12" t="s">
         <v>91</v>
@@ -19961,7 +19961,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B18" s="12" t="s">
         <v>93</v>
@@ -19976,7 +19976,7 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>95</v>
@@ -19991,7 +19991,7 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>97</v>
@@ -20006,7 +20006,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>99</v>
@@ -20021,7 +20021,7 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>101</v>
@@ -20036,7 +20036,7 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>237</v>
@@ -20051,7 +20051,7 @@
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>239</v>
@@ -20066,7 +20066,7 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>209</v>
@@ -20081,7 +20081,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>119</v>
@@ -20096,7 +20096,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>195</v>
@@ -20111,7 +20111,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>197</v>
@@ -20126,7 +20126,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>199</v>
@@ -20141,7 +20141,7 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>241</v>
@@ -20156,7 +20156,7 @@
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>193</v>
@@ -20171,7 +20171,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B32" s="12" t="s">
         <v>117</v>
@@ -20186,7 +20186,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B33" s="12" t="s">
         <v>249</v>
@@ -20201,7 +20201,7 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>128</v>
@@ -20216,7 +20216,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B35" s="12" t="s">
         <v>251</v>
@@ -20231,7 +20231,7 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B36" s="12" t="s">
         <v>214</v>
@@ -20246,7 +20246,7 @@
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B37" s="12" t="s">
         <v>212</v>
@@ -20261,7 +20261,7 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B38" s="12" t="s">
         <v>130</v>
@@ -20276,7 +20276,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B39" s="12" t="s">
         <v>132</v>
@@ -20291,7 +20291,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B40" s="12" t="s">
         <v>134</v>
@@ -20306,7 +20306,7 @@
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>137</v>
@@ -20321,7 +20321,7 @@
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B42" s="12" t="s">
         <v>139</v>
@@ -20336,7 +20336,7 @@
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B43" s="12" t="s">
         <v>141</v>
@@ -20351,7 +20351,7 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B44" s="12" t="s">
         <v>143</v>
@@ -20366,7 +20366,7 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B45" s="12" t="s">
         <v>145</v>
@@ -20381,7 +20381,7 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B46" s="12" t="s">
         <v>147</v>
@@ -20396,7 +20396,7 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>149</v>
@@ -20411,7 +20411,7 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>217</v>
@@ -20426,7 +20426,7 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>151</v>
@@ -20441,7 +20441,7 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B50" s="12" t="s">
         <v>153</v>
@@ -20456,7 +20456,7 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B51" s="12" t="s">
         <v>155</v>
@@ -20471,7 +20471,7 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B52" s="12" t="s">
         <v>157</v>
@@ -20486,7 +20486,7 @@
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B53" s="12" t="s">
         <v>159</v>
@@ -20501,7 +20501,7 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B54" s="12" t="s">
         <v>161</v>
@@ -20516,7 +20516,7 @@
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>163</v>
@@ -20531,7 +20531,7 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>165</v>
@@ -20546,7 +20546,7 @@
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B57" s="12" t="s">
         <v>167</v>
@@ -20561,7 +20561,7 @@
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B58" s="12" t="s">
         <v>169</v>
@@ -20576,7 +20576,7 @@
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B59" s="12" t="s">
         <v>171</v>
@@ -20591,7 +20591,7 @@
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B60" s="12" t="s">
         <v>173</v>
@@ -20606,7 +20606,7 @@
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B61" s="12" t="s">
         <v>175</v>
@@ -20621,7 +20621,7 @@
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B62" s="12" t="s">
         <v>219</v>
@@ -20636,7 +20636,7 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B63" s="12" t="s">
         <v>221</v>
@@ -20651,7 +20651,7 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B64" s="12" t="s">
         <v>223</v>
@@ -20666,7 +20666,7 @@
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B65" s="12" t="s">
         <v>225</v>
@@ -20681,7 +20681,7 @@
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B66" s="12" t="s">
         <v>235</v>
@@ -20696,7 +20696,7 @@
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B67" s="12" t="s">
         <v>227</v>
@@ -20711,7 +20711,7 @@
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B68" s="12" t="s">
         <v>229</v>
@@ -20726,7 +20726,7 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B69" s="12" t="s">
         <v>231</v>
@@ -20741,7 +20741,7 @@
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B70" s="12" t="s">
         <v>233</v>
@@ -20756,7 +20756,7 @@
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B71" s="12" t="s">
         <v>177</v>

</xml_diff>